<commit_message>
Update Matrixport balance report
Latest comparison run: all 3 tokens (TRX, USDT, USDC) match between API and DAM portfolio.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/matrixport_balance.xlsx
+++ b/matrixport_balance.xlsx
@@ -33,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -48,6 +48,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001E6B3C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007B2D8B"/>
       </patternFill>
     </fill>
     <fill>
@@ -74,7 +79,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -82,7 +87,10 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -448,11 +456,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -466,6 +476,16 @@
           <t>Available Balance</t>
         </is>
       </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Balance</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Frozen Balance</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -476,6 +496,12 @@
       <c r="B2" t="n">
         <v>1.698296768198783</v>
       </c>
+      <c r="C2" t="n">
+        <v>1.698296768198783</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -486,6 +512,12 @@
       <c r="B3" t="n">
         <v>5</v>
       </c>
+      <c r="C3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -495,6 +527,12 @@
       </c>
       <c r="B4" t="n">
         <v>20.06</v>
+      </c>
+      <c r="C4" t="n">
+        <v>20.06</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -508,40 +546,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="23" customWidth="1" min="3" max="3"/>
     <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Currency</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Product Type</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>Balance</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>Interest</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Balance (USD)</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Interest (USD)</t>
         </is>
       </c>
     </row>
@@ -557,13 +601,16 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.1000002095152897</v>
+        <v>0.1000003255812135</v>
       </c>
       <c r="D2" t="n">
-        <v>4.2327714072878e-05</v>
+        <v>4.2443779996593e-05</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0999747364619199</v>
+        <v>0.09997616950256605</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4.243352727709702e-05</v>
       </c>
     </row>
   </sheetData>
@@ -577,38 +624,44 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Account</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Token</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Price (24H)</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Total Amount</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Value (USD)</t>
         </is>
@@ -617,64 +670,79 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>USDT</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>0.9998</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>+0.020%</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>1.798296768198783</v>
+          <t>David New BIT Account</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>TRX</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0.34939515</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>+1.187%</t>
+        </is>
       </c>
       <c r="E2" t="n">
-        <v>1.797937108845143</v>
+        <v>5</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1.74697575</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>USDC</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>0.9998</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>+0.020%</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>20.06</v>
+          <t>David New BIT Account</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>USDT</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0.9997</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>+0.000%</t>
+        </is>
       </c>
       <c r="E3" t="n">
-        <v>20.055988</v>
+        <v>1.798296768198783</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1.797757279168324</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TRX</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>0.35082982</v>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>+1.681%</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>5</v>
+          <t>David New BIT Account</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>USDC</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0.9997</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>+0.000%</t>
+        </is>
       </c>
       <c r="E4" t="n">
-        <v>1.7541491</v>
+        <v>20.06</v>
+      </c>
+      <c r="F4" t="n">
+        <v>20.053982</v>
       </c>
     </row>
   </sheetData>
@@ -688,191 +756,212 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="21" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
     <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="19" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Account</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Token</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Balance API</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Balance+ API</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Total API Balance</t>
-        </is>
-      </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Total API</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>DAM Total Amount</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Difference</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Match</t>
-        </is>
-      </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
           <t>DAM Price</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>DAM Price (24H)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>DAM Value (USD)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>David New BIT Account</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>TRX</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>0.34939515</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>+1.187%</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="n">
+        <v>1.746976</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>David New BIT Account</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>USDT</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="C3" s="4" t="n">
         <v>1.69829677</v>
       </c>
-      <c r="C2" s="3" t="n">
-        <v>0.10000021</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>1.79829698</v>
-      </c>
-      <c r="E2" s="3" t="n">
+      <c r="D3" s="4" t="n">
+        <v>0.10000033</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>1.79829709</v>
+      </c>
+      <c r="F3" s="4" t="n">
         <v>1.79829677</v>
       </c>
-      <c r="F2" s="3" t="n">
-        <v>2.1e-07</v>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>✅ Match</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>0.99980000</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>+0.020%</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="n">
-        <v>1.797937</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="G3" s="4" t="n">
+        <v>3.3e-07</v>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>0.99970000</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>+0.000%</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>1.797757</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>David New BIT Account</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
         <is>
           <t>USDC</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="C4" s="4" t="n">
         <v>20.06</v>
       </c>
-      <c r="C3" s="3" t="n">
+      <c r="D4" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="E4" s="4" t="n">
         <v>20.06</v>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="F4" s="4" t="n">
         <v>20.06</v>
       </c>
-      <c r="F3" s="3" t="n">
+      <c r="G4" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>✅ Match</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>0.99980000</t>
-        </is>
-      </c>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>+0.020%</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="n">
-        <v>20.055988</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>TRX</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>✅ Match</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>0.35082982</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>+1.681%</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="n">
-        <v>1.754149</v>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>MATCH</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>0.99970000</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>+0.000%</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>20.053982</v>
       </c>
     </row>
   </sheetData>

</xml_diff>